<commit_message>
Update dashboard, data, and deployment assets
</commit_message>
<xml_diff>
--- a/Raw Data Oil Company.xlsx
+++ b/Raw Data Oil Company.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halea\Nextcloud\Documents\Petroleum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5657200-FDC8-4E2B-BE7D-540A9D2C31DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8E068D-3CCA-41B4-BF52-1EE793874C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="8" xr2:uid="{2321E7CB-9D14-4AF8-907B-0A622BD8B578}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="4" activeTab="4" xr2:uid="{2321E7CB-9D14-4AF8-907B-0A622BD8B578}"/>
   </bookViews>
   <sheets>
     <sheet name="Actual_Company2 Tongatapu" sheetId="1" r:id="rId1"/>
@@ -540,9 +540,6 @@
     <xf numFmtId="164" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -559,9 +556,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -627,39 +621,45 @@
     <xf numFmtId="164" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -999,28 +999,29 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="10" width="8" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42" t="s">
+      <c r="B1" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42" t="s">
+      <c r="E1" s="39"/>
+      <c r="F1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="43"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
@@ -1550,72 +1551,144 @@
         <f t="shared" si="0"/>
         <v>46119</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+      <c r="B24" s="8">
+        <v>400893</v>
+      </c>
+      <c r="C24" s="8">
+        <v>99700</v>
+      </c>
+      <c r="D24" s="8">
+        <v>252748</v>
+      </c>
+      <c r="E24" s="8">
+        <v>61400</v>
+      </c>
+      <c r="F24" s="8">
+        <v>250338</v>
+      </c>
+      <c r="G24" s="8">
+        <v>18900</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <f t="shared" si="0"/>
         <v>46120</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
+      <c r="B25" s="9">
+        <v>345157</v>
+      </c>
+      <c r="C25" s="9">
+        <v>55400</v>
+      </c>
+      <c r="D25" s="9">
+        <v>217109</v>
+      </c>
+      <c r="E25" s="9">
+        <v>35700</v>
+      </c>
+      <c r="F25" s="9">
+        <v>228309</v>
+      </c>
+      <c r="G25" s="9">
+        <v>22700</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6">
         <f t="shared" si="0"/>
         <v>46121</v>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+      <c r="B26" s="8">
+        <v>283388</v>
+      </c>
+      <c r="C26" s="8">
+        <v>71600</v>
+      </c>
+      <c r="D26" s="8">
+        <v>193741</v>
+      </c>
+      <c r="E26" s="8">
+        <v>23730</v>
+      </c>
+      <c r="F26" s="8">
+        <v>209082</v>
+      </c>
+      <c r="G26" s="8">
+        <v>18900</v>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <f t="shared" si="0"/>
         <v>46122</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+      <c r="B27" s="8">
+        <v>1000506</v>
+      </c>
+      <c r="C27" s="8">
+        <v>69200</v>
+      </c>
+      <c r="D27" s="8">
+        <v>562852</v>
+      </c>
+      <c r="E27" s="8">
+        <v>31600</v>
+      </c>
+      <c r="F27" s="8">
+        <v>505156</v>
+      </c>
+      <c r="G27" s="8">
+        <v>1000</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <f t="shared" si="0"/>
         <v>46123</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
+      <c r="B28" s="8">
+        <v>1000506</v>
+      </c>
+      <c r="C28" s="8">
+        <v>0</v>
+      </c>
+      <c r="D28" s="8">
+        <v>562852</v>
+      </c>
+      <c r="E28" s="8">
+        <v>0</v>
+      </c>
+      <c r="F28" s="8">
+        <v>505156</v>
+      </c>
+      <c r="G28" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <f t="shared" si="0"/>
         <v>46124</v>
       </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
+      <c r="B29" s="8">
+        <v>1000506</v>
+      </c>
+      <c r="C29" s="8">
+        <v>0</v>
+      </c>
+      <c r="D29" s="8">
+        <v>562852</v>
+      </c>
+      <c r="E29" s="8">
+        <v>0</v>
+      </c>
+      <c r="F29" s="8">
+        <v>505156</v>
+      </c>
+      <c r="G29" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
@@ -1687,39 +1760,40 @@
   <dimension ref="A2:H36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="8" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.25">
       <c r="D2" s="10"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.25">
       <c r="A3" s="10"/>
-      <c r="B3" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="13" t="s">
+      <c r="B3" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="14"/>
+      <c r="E3" s="46"/>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="17" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2105,60 +2179,108 @@
         <f t="shared" si="0"/>
         <v>46119</v>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
+      <c r="B26" s="8">
+        <v>330227</v>
+      </c>
+      <c r="C26" s="8">
+        <v>9000</v>
+      </c>
+      <c r="D26" s="8">
+        <v>235313</v>
+      </c>
+      <c r="E26" s="8">
+        <v>6000</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <f t="shared" si="0"/>
         <v>46120</v>
       </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
+      <c r="B27" s="9">
+        <v>317077</v>
+      </c>
+      <c r="C27" s="9">
+        <v>13000</v>
+      </c>
+      <c r="D27" s="9">
+        <v>232250</v>
+      </c>
+      <c r="E27" s="9">
+        <v>3000</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <f t="shared" si="0"/>
         <v>46121</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="B28" s="8">
+        <v>317026</v>
+      </c>
+      <c r="C28" s="8">
+        <v>0</v>
+      </c>
+      <c r="D28" s="8">
+        <v>231976</v>
+      </c>
+      <c r="E28" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <f t="shared" si="0"/>
         <v>46122</v>
       </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
+      <c r="B29" s="8">
+        <v>308594</v>
+      </c>
+      <c r="C29" s="8">
+        <v>8000</v>
+      </c>
+      <c r="D29" s="8">
+        <v>227253</v>
+      </c>
+      <c r="E29" s="8">
+        <v>2500</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <f t="shared" si="0"/>
         <v>46123</v>
       </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="B30" s="8">
+        <v>308594</v>
+      </c>
+      <c r="C30" s="8">
+        <v>0</v>
+      </c>
+      <c r="D30" s="8">
+        <v>227253</v>
+      </c>
+      <c r="E30" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <f t="shared" si="0"/>
         <v>46124</v>
       </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
+      <c r="B31" s="8">
+        <v>308594</v>
+      </c>
+      <c r="C31" s="8">
+        <v>0</v>
+      </c>
+      <c r="D31" s="8">
+        <v>227253</v>
+      </c>
+      <c r="E31" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
@@ -2231,42 +2353,42 @@
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="10"/>
-      <c r="B1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="13" t="s">
+      <c r="B1" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="50"/>
+      <c r="D1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="14"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="46"/>
     </row>
     <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
-      <c r="L2" s="19"/>
+      <c r="L2" s="18"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
@@ -2277,7 +2399,7 @@
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
-      <c r="G3" s="22">
+      <c r="G3" s="20">
         <f>SUM(E3:F3)</f>
         <v>0</v>
       </c>
@@ -2292,7 +2414,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="7"/>
-      <c r="G4" s="22">
+      <c r="G4" s="20">
         <f t="shared" ref="G4:G34" si="0">SUM(E4:F4)</f>
         <v>0</v>
       </c>
@@ -2307,7 +2429,7 @@
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="7"/>
-      <c r="G5" s="22">
+      <c r="G5" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2322,7 +2444,7 @@
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="22">
+      <c r="G6" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2337,7 +2459,7 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="23">
+      <c r="G7" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2352,7 +2474,7 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="23">
+      <c r="G8" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2367,7 +2489,7 @@
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
-      <c r="G9" s="23">
+      <c r="G9" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2382,7 +2504,7 @@
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
-      <c r="G10" s="23">
+      <c r="G10" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2397,7 +2519,7 @@
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="23">
+      <c r="G11" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2412,7 +2534,7 @@
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
-      <c r="G12" s="23">
+      <c r="G12" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2427,7 +2549,7 @@
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
-      <c r="G13" s="23">
+      <c r="G13" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2442,7 +2564,7 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
-      <c r="G14" s="23">
+      <c r="G14" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2457,7 +2579,7 @@
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
-      <c r="G15" s="23">
+      <c r="G15" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2472,7 +2594,7 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="23">
+      <c r="G16" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2498,7 +2620,7 @@
         <f>84910-20000</f>
         <v>64910</v>
       </c>
-      <c r="G17" s="23">
+      <c r="G17" s="21">
         <f t="shared" si="0"/>
         <v>84910</v>
       </c>
@@ -2524,7 +2646,7 @@
         <f>121010-68000</f>
         <v>53010</v>
       </c>
-      <c r="G18" s="23">
+      <c r="G18" s="21">
         <f t="shared" si="0"/>
         <v>121010</v>
       </c>
@@ -2550,7 +2672,7 @@
         <f>142000-80000</f>
         <v>62000</v>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="21">
         <f t="shared" si="0"/>
         <v>142000</v>
       </c>
@@ -2575,7 +2697,7 @@
       <c r="F20" s="8">
         <v>0</v>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2600,7 +2722,7 @@
       <c r="F21" s="8">
         <v>4000</v>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="21">
         <f t="shared" si="0"/>
         <v>44000</v>
       </c>
@@ -2625,7 +2747,7 @@
       <c r="F22" s="9">
         <v>0</v>
       </c>
-      <c r="G22" s="23">
+      <c r="G22" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2650,7 +2772,7 @@
       <c r="F23" s="8">
         <v>0</v>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="21">
         <f t="shared" si="0"/>
         <v>100010</v>
       </c>
@@ -2665,7 +2787,7 @@
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
-      <c r="G24" s="23">
+      <c r="G24" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2680,7 +2802,7 @@
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
-      <c r="G25" s="23">
+      <c r="G25" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2695,7 +2817,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
-      <c r="G26" s="23">
+      <c r="G26" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2710,7 +2832,7 @@
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
-      <c r="G27" s="23">
+      <c r="G27" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2725,7 +2847,7 @@
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
-      <c r="G28" s="23">
+      <c r="G28" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2740,7 +2862,7 @@
       <c r="D29" s="8"/>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
-      <c r="G29" s="23">
+      <c r="G29" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2755,7 +2877,7 @@
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
-      <c r="G30" s="23">
+      <c r="G30" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2770,7 +2892,7 @@
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
-      <c r="G31" s="23">
+      <c r="G31" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2785,7 +2907,7 @@
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
-      <c r="G32" s="23">
+      <c r="G32" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2800,7 +2922,7 @@
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
-      <c r="G33" s="23">
+      <c r="G33" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2815,7 +2937,7 @@
       <c r="D34" s="8"/>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
-      <c r="G34" s="23">
+      <c r="G34" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2841,68 +2963,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="24"/>
-      <c r="C1" s="25" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="27" t="s">
+      <c r="D1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="25" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="29">
+      <c r="C2" s="27">
         <v>46136</v>
       </c>
-      <c r="D2" s="30">
+      <c r="D2" s="28">
         <v>150000</v>
       </c>
-      <c r="E2" s="30">
+      <c r="E2" s="28">
         <v>700000</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="31">
+      <c r="C3" s="29">
         <v>46155</v>
       </c>
-      <c r="D3" s="32">
+      <c r="D3" s="30">
         <v>150000</v>
       </c>
-      <c r="E3" s="32">
+      <c r="E3" s="30">
         <v>700000</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2919,80 +3041,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1" s="24"/>
-      <c r="C1" s="25" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="26" t="s">
+      <c r="D1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="25" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="29">
+      <c r="C2" s="27">
         <v>46107</v>
       </c>
-      <c r="D2" s="30">
+      <c r="D2" s="28">
         <v>807300</v>
       </c>
-      <c r="E2" s="30">
+      <c r="E2" s="28">
         <v>384000</v>
       </c>
-      <c r="F2" s="32">
+      <c r="F2" s="30">
         <v>177800</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="31">
+      <c r="C3" s="29">
         <v>46118</v>
       </c>
-      <c r="D3" s="30">
+      <c r="D3" s="28">
         <v>807300</v>
       </c>
-      <c r="E3" s="30">
+      <c r="E3" s="28">
         <v>396000</v>
       </c>
-      <c r="F3" s="32">
+      <c r="F3" s="30">
         <v>292100</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="32"/>
+      <c r="C4" s="29">
+        <v>46134</v>
+      </c>
+      <c r="D4" s="28">
+        <v>759000</v>
+      </c>
+      <c r="E4" s="28">
+        <v>556600</v>
+      </c>
+      <c r="F4" s="30">
+        <v>254000</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="32"/>
+      <c r="C5" s="29">
+        <v>46145</v>
+      </c>
+      <c r="D5" s="28">
+        <v>772800</v>
+      </c>
+      <c r="E5" s="28">
+        <v>411400</v>
+      </c>
+      <c r="F5" s="30">
+        <v>190500</v>
+      </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="32"/>
+      <c r="C6" s="29">
+        <v>46158</v>
+      </c>
+      <c r="D6" s="28">
+        <v>841800</v>
+      </c>
+      <c r="E6" s="28">
+        <v>496100</v>
+      </c>
+      <c r="F6" s="30">
+        <v>228600</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3004,67 +3150,79 @@
   <dimension ref="B1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="24"/>
-      <c r="C1" s="25" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="27" t="s">
+      <c r="D1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="25" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="29">
+      <c r="C2" s="27">
         <v>46115</v>
       </c>
-      <c r="D2" s="30">
+      <c r="D2" s="28">
         <v>303600</v>
       </c>
-      <c r="E2" s="30">
+      <c r="E2" s="28">
         <v>132000</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
+      <c r="C3" s="29">
+        <v>46144</v>
+      </c>
+      <c r="D3" s="28">
+        <v>220800</v>
+      </c>
+      <c r="E3" s="28">
+        <v>169400</v>
+      </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
+      <c r="C4" s="29">
+        <v>46169</v>
+      </c>
+      <c r="D4" s="28">
+        <v>234600</v>
+      </c>
+      <c r="E4" s="28">
+        <v>181500</v>
+      </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3082,18 +3240,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C1" s="24"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="41" t="s">
+      <c r="C1" s="22"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="42"/>
-      <c r="G1" s="43"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C2" s="33"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="35" t="s">
+      <c r="C2" s="31"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="33" t="s">
         <v>16</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -3104,55 +3262,55 @@
       </c>
     </row>
     <row r="3" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="36">
+      <c r="E3" s="34">
         <v>1223106</v>
       </c>
-      <c r="F3" s="36">
+      <c r="F3" s="34">
         <v>858361</v>
       </c>
-      <c r="G3" s="36">
+      <c r="G3" s="34">
         <v>589571</v>
       </c>
     </row>
     <row r="4" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="37">
+      <c r="E4" s="35">
         <v>47000</v>
       </c>
-      <c r="F4" s="37">
+      <c r="F4" s="35">
         <v>45000</v>
       </c>
-      <c r="G4" s="37">
+      <c r="G4" s="35">
         <v>24500</v>
       </c>
     </row>
     <row r="5" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="36">
         <f>E3-E4</f>
         <v>1176106</v>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="36">
         <f>F3-F4</f>
         <v>813361</v>
       </c>
-      <c r="G5" s="38">
+      <c r="G5" s="36">
         <f>G3-G4</f>
         <v>565071</v>
       </c>
@@ -3168,63 +3326,63 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C1" s="24"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="44" t="s">
+      <c r="C1" s="22"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="46"/>
+      <c r="F1" s="13"/>
     </row>
     <row r="2" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C2" s="33"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="39" t="s">
+      <c r="C2" s="31"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="37">
+      <c r="E3" s="35">
         <v>357582</v>
       </c>
-      <c r="F3" s="37">
+      <c r="F3" s="35">
         <v>289500</v>
       </c>
     </row>
     <row r="4" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="37">
+      <c r="E4" s="35">
         <v>26800</v>
       </c>
-      <c r="F4" s="37">
+      <c r="F4" s="35">
         <v>16165</v>
       </c>
     </row>
     <row r="5" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="36">
         <f>E3-E4</f>
         <v>330782</v>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="36">
         <f>F3-F4</f>
         <v>273335</v>
       </c>
@@ -3246,91 +3404,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="24"/>
-      <c r="B1" s="28"/>
-      <c r="C1" s="11" t="s">
+      <c r="A1" s="22"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="14"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="33"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="39" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="37">
+      <c r="C3" s="35">
         <v>325936</v>
       </c>
-      <c r="D3" s="37">
+      <c r="D3" s="35">
         <v>1832778</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="37">
+      <c r="C4" s="35">
         <v>16085</v>
       </c>
-      <c r="D4" s="37">
+      <c r="D4" s="35">
         <f>46571+26000</f>
         <v>72571</v>
       </c>
-      <c r="E4" s="33"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="36">
         <f>C3-C4</f>
         <v>309851</v>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="36">
         <f>D3-D4</f>
         <v>1760207</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E6" s="28"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E7" s="28"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>